<commit_message>
v2: add §288 Abs. 2 exemption triggers to checklist (13 items marked C)
</commit_message>
<xml_diff>
--- a/v2/output/checklist.xlsx
+++ b/v2/output/checklist.xlsx
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>147</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -5323,10 +5323,14 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of raw materials and supplies costs is disclosed</t>
@@ -5372,10 +5376,14 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I33" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of merchandise costs is disclosed</t>
@@ -5421,10 +5429,14 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of purchased services costs is disclosed</t>
@@ -5470,10 +5482,14 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of Löhne und Gehälter is disclosed</t>
@@ -5519,10 +5535,14 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of social security and pension costs is disclosed</t>
@@ -5568,10 +5588,14 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
           <t>Verify average number of employees is disclosed</t>
@@ -6412,7 +6436,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -6612,7 +6636,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -6665,7 +6689,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -7110,7 +7134,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -7310,7 +7334,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -7701,10 +7725,14 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>Verify detailed breakdown of revenue by type of business activity</t>
@@ -7848,10 +7876,14 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
           <t>Verify disclosure of government grants received and their accounting treatment</t>
@@ -14156,10 +14188,14 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I94" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of raw materials and supplies costs is disclosed</t>
@@ -14205,10 +14241,14 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I95" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of merchandise costs is disclosed</t>
@@ -14254,10 +14294,14 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I96" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of purchased services costs is disclosed</t>
@@ -14303,10 +14347,14 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I97" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of Löhne und Gehälter is disclosed</t>
@@ -14352,10 +14400,14 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I98" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
           <t>Verify breakdown of social security and pension costs is disclosed</t>
@@ -14401,10 +14453,14 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I99" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
           <t>Verify average number of employees is disclosed</t>
@@ -15161,7 +15217,7 @@
       </c>
       <c r="I114" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J114" s="3" t="inlineStr">
@@ -15361,7 +15417,7 @@
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J118" s="3" t="inlineStr">
@@ -15414,7 +15470,7 @@
       </c>
       <c r="I119" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J119" s="3" t="inlineStr">
@@ -15859,7 +15915,7 @@
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J128" s="3" t="inlineStr">
@@ -16059,7 +16115,7 @@
       </c>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>Entity invokes §288 Abs. 2 exemption</t>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
         </is>
       </c>
       <c r="J132" s="3" t="inlineStr">
@@ -16450,10 +16506,14 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I140" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J140" s="3" t="inlineStr">
         <is>
           <t>Verify detailed breakdown of revenue by type of business activity</t>
@@ -16597,10 +16657,14 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I143" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>Exempt for medium GmbH per §288 Abs. 2 HGB - not required to disclose</t>
+        </is>
+      </c>
       <c r="J143" s="3" t="inlineStr">
         <is>
           <t>Verify disclosure of government grants received and their accounting treatment</t>

</xml_diff>